<commit_message>
Enforce validation for code fields
Add uppercase, character, and 100-character validation for code fields across UI inputs, API payloads, and spreadsheet imports while preserving ordinary text. Update related import templates and developer documentation.
</commit_message>
<xml_diff>
--- a/download/netrent-contract-import-template.xlsx
+++ b/download/netrent-contract-import-template.xlsx
@@ -399,16 +399,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J4"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="24.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="10" max="10" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -463,7 +463,7 @@
         <v>1</v>
       </c>
       <c r="G2" t="str">
-        <v>THB</v>
+        <v>USD</v>
       </c>
       <c r="H2" t="str">
         <v>ACTIVE</v>
@@ -495,7 +495,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="str">
-        <v>THB</v>
+        <v>USD</v>
       </c>
       <c r="H3" t="str">
         <v>ACTIVE</v>
@@ -527,7 +527,7 @@
         <v>0</v>
       </c>
       <c r="G4" t="str">
-        <v>THB</v>
+        <v>USD</v>
       </c>
       <c r="H4" t="str">
         <v>DRAFT</v>

</xml_diff>